<commit_message>
Governanca: detalhar cenarios aprovados de divergencia BK-005
O que é: documentação e rastreamento dos exemplos da decisão C-01 para pagamentos divergentes.

O que foi feito: detalhei os casos de diferença de qualquer valor, inclusive R$ 0,01; mantive títulos sem baixa até análise; documentei tratamento de descontos, tarifas, estornos, vínculos ambíguos, auditoria e reprocessamento sem duplicidade. Sincronizei backlog, decisão, visão geral, planilha, prévias e manifesto. Nenhuma tela, regra aprovada ou código do produto foi alterado; testes do projeto não foram executados.

Próximo passo: aguardar o documento atualizado da calculadora para fechar a regra da reserva sugerida e seguir BK-006.

Quanto falta da tarefa BK-005: 0% (100% concluída no escopo documental).

Quanto falta do projeto: 95,3% por contagem simples do rastreador (6 de 127 concluídas); 124 tarefas ainda aguardam auditoria e três conclusões históricas não foram revalidadas. Não é uma medida real de esforço ou prontidão.
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R85e2635a033c4b24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Raf559c0e99b345ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R6add47113ffe49db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R2525127df7c94921"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R3aed19cbe7cf4e93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R2d7d84cd81c64b61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Rc9fc4934fc7d417e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Raa5736e6a1d6402f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -554,7 +554,7 @@
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>Status atualizado em 11/10/2026 | fechamento funcional de 13/09/2026</x:v>
+        <x:v>Status atualizado em 10/10/2026 | fechamento funcional de 13/09/2026</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -632,7 +632,7 @@
       </x:c>
       <x:c r="B7" s="22" t="n">
         <x:f>COUNTIFS('Tarefas'!$D$6:$D$132,"Planejamento",'Tarefas'!$G$6:$G$132,1)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C7" s="11" t="inlineStr">
         <x:is>
@@ -660,7 +660,7 @@
       </x:c>
       <x:c r="B8" s="27" t="n">
         <x:f>SUM('Tarefas'!$M$6:$M$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.03937007874015748</x:v>
+        <x:v>0.047244094488188976</x:v>
       </x:c>
       <x:c r="C8" s="11" t="inlineStr">
         <x:is>
@@ -815,7 +815,7 @@
       </x:c>
       <x:c r="C14" s="28" t="n">
         <x:f>SUMIFS('Tarefas'!$M$6:$M$132,'Tarefas'!$B$6:$B$132,A14)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A14)</x:f>
-        <x:v>0.3125</x:v>
+        <x:v>0.375</x:v>
       </x:c>
       <x:c r="D14" s="2" t="n"/>
       <x:c r="E14" s="2" t="inlineStr">
@@ -1176,7 +1176,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>BK-000 e BK-004 auditadas em 10–11/10; 125 tarefas ainda aguardam revisão. Regra definida não equivale a implementação concluída.</x:v>
+        <x:v>BK-000, BK-004 e BK-005 auditadas nesta rodada; 124 tarefas ainda aguardam revisão. Regra definida não equivale a implementação concluída.</x:v>
       </x:c>
       <x:c r="B33" s="2" t="n"/>
       <x:c r="C33" s="2" t="n"/>
@@ -1662,16 +1662,18 @@
         <x:v>Planejamento</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Concluída</x:v>
       </x:c>
       <x:c r="F11" s="30" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G11" s="32" t="n">
         <x:f>IF(AND(E11="Concluída",H11&lt;&gt;""),1,0)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H11" s="12" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H11" s="12" t="str">
+        <x:v>Cenários de aceite e tratamento de ambiguidade registrados nesta tarefa a partir da regra C-01 aprovada; não houve alteração de código nem execução de testes.</x:v>
+      </x:c>
       <x:c r="I11" s="11" t="str">
         <x:v>Majucau / Financeiro</x:v>
       </x:c>
@@ -1684,7 +1686,7 @@
       </x:c>
       <x:c r="M11" s="11" t="n">
         <x:f>F11*G11</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="72" customHeight="1">
@@ -6575,7 +6577,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbadaebe5b9749f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c84d42adf1c4a4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6927,7 +6929,7 @@
         <x:v>Aplicar a definição vigente; execução, evidência e aceite são registrados nas tarefas relacionadas.</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
-        <x:v>Marcar divergência e manter o título sem baixa até a análise. Casos complementares serão detalhados em BK-005.</x:v>
+        <x:v>Qualquer diferença, inclusive R$ 0,01, marca divergência e mantém o título sem baixa até análise. Cenários de aceite, tratamento de ambiguidade e proteção contra duplicidade estão detalhados em BK-005.</x:v>
       </x:c>
       <x:c r="G14" s="10" t="str">
         <x:v>C_Conflitos!A3:L3; Fechamento das questões ainda tratadas como abertas — 13/09/2026</x:v>
@@ -9808,7 +9810,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f77f6f26ffc4123"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6416207027934f65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10457,7 +10459,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rced378c258b24ae6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a2944d3c0214580"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Governança: atualizar auditorias BK-001 e BK-002
O que é: revalidar o inventário de materiais e o ponto de partida no GitHub.

O que foi feito: registrei que não há outro clone, servidor ou ambiente de trabalho fora deste checkout; atualizei evidência, backlog, planilha, prévias e hashes do manifesto. BK-001 segue aberta porque os arquivos originais não estão no arquivo privado e falta decidir se serão enviados ou se hashes e extrações bastam. Nenhuma tela ou regra de negócio foi alterada; testes não foram executados.

Próximo passo: aguardar a decisão sobre os originais da BK-001; então continuar a revisão das tarefas dependentes.

Quanto falta da meta para terminar a tarefa: BK-002, 0%; BK-001 continua pendente dessa decisão.

Quanto falta da meta para terminar o projeto: 96,1% por contagem do rastreador (122 de 127 tarefas não concluídas). Esse número não mede prontidão real; ainda não há prazo confiável.
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R3aed19cbe7cf4e93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R2d7d84cd81c64b61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Rc9fc4934fc7d417e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Raa5736e6a1d6402f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R4e199a25579d45ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Rdf85e673887d4172"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R3ac31b6bf8e74a30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rb516162f4b5842f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -632,7 +632,7 @@
       </x:c>
       <x:c r="B7" s="22" t="n">
         <x:f>COUNTIFS('Tarefas'!$D$6:$D$132,"Planejamento",'Tarefas'!$G$6:$G$132,1)</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C7" s="11" t="inlineStr">
         <x:is>
@@ -660,7 +660,7 @@
       </x:c>
       <x:c r="B8" s="27" t="n">
         <x:f>SUM('Tarefas'!$M$6:$M$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.047244094488188976</x:v>
+        <x:v>0.03937007874015748</x:v>
       </x:c>
       <x:c r="C8" s="11" t="inlineStr">
         <x:is>
@@ -815,7 +815,7 @@
       </x:c>
       <x:c r="C14" s="28" t="n">
         <x:f>SUMIFS('Tarefas'!$M$6:$M$132,'Tarefas'!$B$6:$B$132,A14)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A14)</x:f>
-        <x:v>0.375</x:v>
+        <x:v>0.3125</x:v>
       </x:c>
       <x:c r="D14" s="2" t="n"/>
       <x:c r="E14" s="2" t="inlineStr">
@@ -1176,7 +1176,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>BK-000, BK-004 e BK-005 auditadas nesta rodada; 124 tarefas ainda aguardam revisão. Regra definida não equivale a implementação concluída.</x:v>
+        <x:v>BK-000, BK-002, BK-004 e BK-005 auditadas; BK-001 aguarda decisão sobre arquivos originais; 122 tarefas aguardam revisão. Regra definida não equivale a implementação concluída.</x:v>
       </x:c>
       <x:c r="B33" s="2" t="n"/>
       <x:c r="C33" s="2" t="n"/>
@@ -1500,29 +1500,31 @@
         <x:v>Planejamento</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
-        <x:v>Concluída</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="F7" s="30" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="32" t="n">
         <x:f>IF(AND(E7="Concluída",H7&lt;&gt;""),1,0)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H7" s="12" t="str">
-        <x:v>MAJUCAU_ANALISE_E_DECISOES_v0.md — inventário e análise; inspeção dos materiais e GitHub nesta sessão. Evidência original preservada na versão 0; esta revisão não altera a conclusão desse levantamento.</x:v>
+        <x:v>Inventário histórico registra 16 PNGs, 15 imagens únicas, 20 abas, T10 duplicada e materiais ausentes; a extração tem 20 entradas de aba e as versões v0/v1/v2 estão preservadas. Os hashes dos originais constam em FONTES.md, mas sources/private/material-original não existe neste checkout e os nomes exatos não foram encontrados em Downloads. A responsável foi consultada se enviará os originais ou aceita hashes/extrações; resposta pendente. BK-001 permanece aberta até a decisão.</x:v>
       </x:c>
       <x:c r="I7" s="11" t="str">
         <x:v>Produto + UX</x:v>
       </x:c>
       <x:c r="J7" s="11" t="str"/>
-      <x:c r="K7" s="11" t="str"/>
+      <x:c r="K7" s="11" t="str">
+        <x:v>Aguardar orientação sobre os originais: envio para arquivo privado local ou aceitação de hashes e extrações como suficientes.</x:v>
+      </x:c>
       <x:c r="L7" s="11" t="str">
-        <x:v>Pacote fornecido; manifesto de arquivos; Consolidação 13/09/2026, consolidação integral; Fechamento vigente 13/09/2026, integral</x:v>
+        <x:v>docs/planejamento/FONTES.md; docs/source/README.md; docs/planejamento/work/source_extract; revision_v1.json; revision_v2.json</x:v>
       </x:c>
       <x:c r="M7" s="11" t="n">
         <x:f>F7*G7</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="72" customHeight="1">
@@ -1549,15 +1551,17 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H8" s="12" t="str">
-        <x:v>MAJUCAU_ANALISE_E_DECISOES_v0.md — inventário e análise; inspeção dos materiais e GitHub nesta sessão. Evidência original preservada na versão 0; esta revisão não altera a conclusão desse levantamento.</x:v>
+        <x:v>Auditoria pública somente de leitura em 10/10/2026: repositório público, branch padrão main no commit 39f8630390936717b2500c8b7ce923dc138cca72; branch de trabalho codex/majucau-artifact-consolidation em b94bb3a, mesma ponta remota, 178 commits à frente e zero atrás de main. A API retornou zero issues e cinco pull requests abertos e não mesclados (#1–#5), todos em outras branches. A afirmação de repositório vazio em v0 é histórica. A responsável confirmou que não há outro clone, servidor ou ambiente de trabalho fora deste checkout; o código é controlado somente pelo Git/GitHub. Nenhuma branch foi mesclada e nenhum teste foi executado.</x:v>
       </x:c>
       <x:c r="I8" s="10" t="str">
         <x:v>Arquitetura</x:v>
       </x:c>
       <x:c r="J8" s="10" t="str"/>
-      <x:c r="K8" s="10" t="str"/>
+      <x:c r="K8" s="10" t="str">
+        <x:v/>
+      </x:c>
       <x:c r="L8" s="10" t="str">
-        <x:v>GitHub majucau /contents e /commits</x:v>
+        <x:v>GitHub REST: repos/guilhermejacyzin/majucau, branches/main, issues?state=all, pulls?state=all; git ls-remote origin; comparação origin/main..HEAD</x:v>
       </x:c>
       <x:c r="M8" s="10" t="n">
         <x:f>F8*G8</x:f>
@@ -6577,7 +6581,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c84d42adf1c4a4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03b99404c46340d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9810,7 +9814,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6416207027934f65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R954bf805c8a14ed8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10459,7 +10463,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a2944d3c0214580"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d93b637c97a4068"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(finance): alinhar mapeamento da calculadora D-003-A
O que é: avanço da especificação técnica da calculadora de aplicação.

O que foi feito: corrigido o Data Dictionary para refletir D-003-A/D-003-C aprovadas; documentado o mapa entre DRE, fluxo diário, reserva e saldo Itaú e as fontes ainda ausentes; atualizado backlog e planilha. Nenhuma tela, regra financeira ou schema foi alterado. Conferências do pacote, fórmulas e backlog passaram.

Próximo passo: identificar o relatório oficial que registra aportes e resgates do principal e, com essa fonte definida, ligar as leituras de produção sem preencher dados ausentes com zero.

Quanto falta da tarefa BK-006: 70% estimados.

Quanto falta da meta do projeto: 92,8% estimados.
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R0b92ed591fed4f99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R41bdbb3be8314419"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R8e748c5c297d43b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Racebe127eac54b99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R3f083ed1f1434dd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Rf13b9a3188c942dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Rc652b006bf9f472d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R2d41f63a62cd481f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.07165354330708662</x:v>
+        <x:v>0.07204724409448819</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -673,7 +673,7 @@
       </x:c>
       <x:c r="C14" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A14)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A14)</x:f>
-        <x:v>0.36562500000000003</x:v>
+        <x:v>0.36875</x:v>
       </x:c>
       <x:c r="D14" s="2"/>
       <x:c r="E14" s="2" t="str">
@@ -1499,9 +1499,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G12" s="16" t="n">
-        <x:v>0.25</x:v>
-      </x:c>
-      <x:c r="H12" s="12" t="str"/>
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="H12" s="12" t="str">
+        <x:v>Mapa em docs/evidence/APPLICATION-RULE-D003A-2026-09-20.md: DRE/fluxo sem ligação de produção; faltam fonte de aportes/resgates e saldo Itaú transferível. Regra e tela preservadas.</x:v>
+      </x:c>
       <x:c r="I12" s="10" t="str">
         <x:v>Majucau / Financeiro</x:v>
       </x:c>
@@ -1518,7 +1520,7 @@
       </x:c>
       <x:c r="N12" s="10" t="n">
         <x:f>F12*G12</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.3</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="72" customHeight="1">
@@ -6732,7 +6734,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d154634219a4a34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re05dce0d27724d71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9943,7 +9945,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1752f7c26284cf9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d4cbfe0312349e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10368,7 +10370,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f1c54c19ce24cb4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R395a79f2e7d44ee4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(security): iniciar mapa de riscos da BK-024
O que é: iniciar o planejamento de segurança e proteção dos dados do Majucau.

O que foi feito: criado um mapa inicial com ativos, caminhos de dados, riscos, controles já encontrados e verificações futuras. Atualizados o backlog estruturado, o documento detalhado, a visão geral e a planilha de evolução. O gerador agora calcula o resumo ponderado pela importância das tarefas e guarda prévias temporárias em artifacts. Nenhuma tela ou regra financeira foi alterada.

Próximo passo: mapear todas as fontes e saídas, completar os controles de acesso, hospedagem, credenciais, retenção e recuperação, e então executar as validações planejadas.

Quantos % da meta falta para terminar a tarefa: 80% da BK-024; os 20% atuais são somente o mapa inicial.

Quantos % da meta falta para terminar o projeto: 92,6% segundo a estimativa atual do backlog, que não mede esforço nem prontidão para produção.
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R3f083ed1f1434dd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Rf13b9a3188c942dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Rc652b006bf9f472d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R2d41f63a62cd481f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rb856a891e9f7496d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R7556482500224e88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R8661690043624694"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rc02c776acf824a25"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -185,7 +185,7 @@
         <x:color rgb="FFA12622"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE4E0"/>
         </x:patternFill>
       </x:fill>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.07204724409448819</x:v>
+        <x:v>0.0736220472440945</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -694,7 +694,7 @@
       </x:c>
       <x:c r="C15" s="25" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A15)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A15)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.022222222222222223</x:v>
       </x:c>
       <x:c r="D15" s="2"/>
       <x:c r="E15" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 11/10/2026: 6 concluídas, 10 em andamento e 111 não iniciadas. Estimativa média: 7,2%; restantes 92,8%. BK-001 aguarda decisão sobre arquivos originais. Regra definida não equivale a implementação concluída.</x:v>
+        <x:v>Backlog em 11/10/2026: 6 concluídas, 11 em andamento e 110 não iniciadas. Estimativa: 7,4%; restante: 92,6%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -2261,15 +2261,17 @@
         <x:v>Desenvolvimento</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="F30" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G30" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H30" s="12" t="str"/>
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="H30" s="12" t="str">
+        <x:v>Mapa inicial em docs/evidence/THREAT-MODEL-INITIAL-2026-10-11.md: ativos, riscos, controles e verificações propostas. Revisão estática, sem testes; falta mapear todas as fontes, implementar controles e validar.</x:v>
+      </x:c>
       <x:c r="I30" s="10" t="str">
         <x:v>Segurança + Arquitetura</x:v>
       </x:c>
@@ -2288,7 +2290,7 @@
       </x:c>
       <x:c r="N30" s="10" t="n">
         <x:f>F30*G30</x:f>
-        <x:v>0</x:v>
+        <x:v>0.2</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="72" customHeight="1">
@@ -6734,7 +6736,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re05dce0d27724d71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b563e57f345464c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9945,7 +9947,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d4cbfe0312349e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fc68f0b44e147b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10370,7 +10372,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R395a79f2e7d44ee4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0d6b7c272a34be9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(security): registrar CI 410 e alinhar BK-024
O que é: registro da evidência de segurança e alinhamento do backlog BK-024.
O que foi feito: documentados os testes controlados de limpeza e a CI #410; alinhados os 30% já registrados no backlog com o JSON e a planilha; manifesto recalculado. Nenhuma tela ou regra financeira foi alterada.
Próximo passo: concluir as demais falhas controladas, fechar o mapa de riscos e validar VM limpa, rede e acesso por perfil.
Quanto falta da tarefa BK-024: 70% (estimativa).
Quanto falta do projeto: 92,6% (estimativa geral do backlog).
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rb856a891e9f7496d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R7556482500224e88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R8661690043624694"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rc02c776acf824a25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R11680138251a46ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R75ffe39dd94e4bde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R358cb6065dc040c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rcffc666f27c94a1b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.0736220472440945</x:v>
+        <x:v>0.07440944881889765</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -694,7 +694,7 @@
       </x:c>
       <x:c r="C15" s="25" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A15)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A15)</x:f>
-        <x:v>0.022222222222222223</x:v>
+        <x:v>0.03333333333333333</x:v>
       </x:c>
       <x:c r="D15" s="2"/>
       <x:c r="E15" s="2" t="str">
@@ -2267,10 +2267,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G30" s="16" t="n">
-        <x:v>0.2</x:v>
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="H30" s="12" t="str">
-        <x:v>Mapa inicial em docs/evidence/THREAT-MODEL-INITIAL-2026-10-11.md: ativos, riscos, controles e verificações propostas. Revisão estática, sem testes; falta mapear todas as fontes, implementar controles e validar.</x:v>
+        <x:v>Falhas controladas securetemp/csvstream e go vet passaram; CI #410 aprovada. Faltam outras falhas, VM limpa, rede e perfis. Detalhes no mapa de riscos.</x:v>
       </x:c>
       <x:c r="I30" s="10" t="str">
         <x:v>Segurança + Arquitetura</x:v>
@@ -2290,7 +2290,7 @@
       </x:c>
       <x:c r="N30" s="10" t="n">
         <x:f>F30*G30</x:f>
-        <x:v>0.2</x:v>
+        <x:v>0.3</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="72" customHeight="1">
@@ -6736,7 +6736,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b563e57f345464c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05283bebfd944f3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9947,7 +9947,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fc68f0b44e147b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4d91f56e6824e2d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10372,7 +10372,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0d6b7c272a34be9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R328b2f0c4b6641b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(governanca): alinhar backlog e calculadora
O que é: Atualizar inventário, evidências do backlog e planilha de governança.
O que foi feito: Corrigida a anotação falsa de que a extração das 20 abas estava ausente; mantida BK-001 pendente porque os 17 arquivos originais ainda faltam. BK-041 foi alinhada a 60% com evidência da falha segura de paginação, sem homologar a resposta real do Bling. A estrutura enviada da calculadora foi registrada como referência aprovada e a planilha de acompanhamento foi regenerada; manifesto validado.
Próximo passo: Receber os originais ou aprovação para usar a extração; responder a dúvida sobre sincronizar apenas o tipo escolhido ou os dois tipos antes de alterar esse comportamento.
Quanto falta da tarefa BK-041: 40%.
Quanto falta do projeto: 92,5%.
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R11680138251a46ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R75ffe39dd94e4bde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R358cb6065dc040c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rcffc666f27c94a1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R9ffa37698abd4b09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R4774c27727de4927"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R86ca7b5283c84d4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R632a0339bb984168"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -185,7 +185,7 @@
         <x:color rgb="FFA12622"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE4E0"/>
         </x:patternFill>
       </x:fill>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.07440944881889765</x:v>
+        <x:v>0.07480314960629922</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -755,7 +755,7 @@
       </x:c>
       <x:c r="C18" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A18)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A18)</x:f>
-        <x:v>0.03666666666666667</x:v>
+        <x:v>0.04</x:v>
       </x:c>
       <x:c r="D18" s="2"/>
       <x:c r="E18" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 11/10/2026: 6 concluídas, 11 em andamento e 110 não iniciadas. Estimativa: 7,4%; restante: 92,6%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 11/10/2026: 6 concluídas, 11 em andamento e 110 não iniciadas. Estimativa: 7,5%; restante: 92,5%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -1282,7 +1282,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H7" s="12" t="str">
-        <x:v>Inventário histórico registra 16 PNGs, 15 imagens únicas, 20 abas, T10 duplicada e materiais ausentes; a extração tem 20 entradas de aba e as versões v0/v1/v2 estão preservadas. Os hashes dos originais constam em FONTES.md, mas sources/private/material-original não existe neste checkout e os nomes exatos não foram encontrados em Downloads. A responsável foi consultada se enviará os originais ou aceita hashes/extrações; resposta pendente. BK-001 permanece aberta até a decisão.</x:v>
+        <x:v>Extração existe em docs/planejamento/work/source_extract/: workbook.json representa 20 abas e manifest.json conserva 17 itens/hashes históricos. Os 17 binários originais não foram localizados; a correspondência da extração não foi comprovada. Aceite aguarda os originais ou aprovação da responsável.</x:v>
       </x:c>
       <x:c r="I7" s="11" t="str">
         <x:v>Produto + UX</x:v>
@@ -1502,7 +1502,7 @@
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="H12" s="12" t="str">
-        <x:v>Mapa em docs/evidence/APPLICATION-RULE-D003A-2026-09-20.md: DRE/fluxo sem ligação de produção; faltam fonte de aportes/resgates e saldo Itaú transferível. Regra e tela preservadas.</x:v>
+        <x:v>Mapa em docs/evidence/APPLICATION-RULE-D003A-2026-09-20.md: DRE/fluxo sem ligação de produção; faltam fonte de aportes/resgates e saldo Itaú transferível. A responsável reiterou em 11/10/2026 que se preserve a estrutura da calculadora enviada; qualquer mapeamento ainda incerto aguarda confirmação. Regra e tela preservadas.</x:v>
       </x:c>
       <x:c r="I12" s="10" t="str">
         <x:v>Majucau / Financeiro</x:v>
@@ -2270,7 +2270,7 @@
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="H30" s="12" t="str">
-        <x:v>Falhas controladas securetemp/csvstream e go vet passaram; CI #410 aprovada. Faltam outras falhas, VM limpa, rede e perfis. Detalhes no mapa de riscos.</x:v>
+        <x:v>Mapa e testes controlados em docs/evidence/THREAT-MODEL-INITIAL-2026-10-11.md. Testes de securetemp/csvstream, go vet e diff check locais passaram; CI #410 passou nos jobs backlog, Windows e PostgreSQL (Go, vet, análise de vulnerabilidades, builds, SBOM, smoke do instalador e consolidação). BK-024 continua em andamento: faltam outras falhas controladas, completar o mapa de riscos e validar VM limpa, rede e acesso por perfil.</x:v>
       </x:c>
       <x:c r="I30" s="10" t="str">
         <x:v>Segurança + Arquitetura</x:v>
@@ -3005,9 +3005,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G47" s="17" t="n">
-        <x:v>0.55</x:v>
-      </x:c>
-      <x:c r="H47" s="12" t="str"/>
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="H47" s="12" t="str">
+        <x:v>60% — filtros de situação por rota e falha segura quando a última página é desconhecida; evidência em docs/evidence/BLING-PAGINATION-CONTRACT-2026-10-11.md. Resposta e cursor da conta real seguem sem homologação.</x:v>
+      </x:c>
       <x:c r="I47" s="11" t="str">
         <x:v>Engenharia</x:v>
       </x:c>
@@ -3026,7 +3028,7 @@
       </x:c>
       <x:c r="N47" s="11" t="n">
         <x:f>F47*G47</x:f>
-        <x:v>0.55</x:v>
+        <x:v>0.6</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="72" customHeight="1">
@@ -6736,7 +6738,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05283bebfd944f3c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb617f7ee2554b23"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9947,7 +9949,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4d91f56e6824e2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae13ae6c7d144eca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10372,7 +10374,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R328b2f0c4b6641b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff57fc35eebc4902"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(seguranca): detalhar auditoria de streaming
O que é: Registrar evidência adicional de streaming e proteção de dados para BK-024.
O que foi feito: Busca estática delimitada confirmou leitura de CSV por linha, respostas do Bling decodificadas em fluxo com limite de 4 MiB/100 registros, consultas de linhas com Rows.Next e limites explícitos nas exceções de leitura completa. Atualizei o mapa de riscos, backlog e planilha; conferi os hashes do manifesto. Nenhuma tela ou regra financeira mudou; não executei testes ou build.
Próximo passo: Completar falhas controladas e validar disco/ACL, VM limpa, rede e perfis; responder a dúvida pendente sobre sincronizar um ou os dois tipos do Bling antes de mudar esse fluxo.
Quanto falta da tarefa BK-024: 70%.
Quanto falta do projeto: 92,5%.
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R9ffa37698abd4b09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R4774c27727de4927"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R86ca7b5283c84d4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R632a0339bb984168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Ra0cce655c164412b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R870396d28d3840e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R9809f63334fe4564"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R8d4ebadb649e41a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2270,7 +2270,7 @@
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="H30" s="12" t="str">
-        <x:v>Mapa e testes controlados em docs/evidence/THREAT-MODEL-INITIAL-2026-10-11.md. Testes de securetemp/csvstream, go vet e diff check locais passaram; CI #410 passou nos jobs backlog, Windows e PostgreSQL (Go, vet, análise de vulnerabilidades, builds, SBOM, smoke do instalador e consolidação). BK-024 continua em andamento: faltam outras falhas controladas, completar o mapa de riscos e validar VM limpa, rede e acesso por perfil.</x:v>
+        <x:v>Mapa e testes controlados em docs/evidence/THREAT-MODEL-INITIAL-2026-10-11.md. Busca estática adicional confirma CSV por linha, Bling com decoder direto e limite de 4 MiB/100 registros por página, e consultas de linhas com Rows.Next(); leituras completas restantes têm limites explícitos. BK-024 permanece em 30% porque ainda faltam falhas controladas, fechar o mapa de riscos e validar VM limpa, rede, disco cheio/ACL e acesso por perfil.</x:v>
       </x:c>
       <x:c r="I30" s="10" t="str">
         <x:v>Segurança + Arquitetura</x:v>
@@ -6738,7 +6738,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb617f7ee2554b23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7758b7ed2a09412c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9949,7 +9949,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae13ae6c7d144eca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf87e6630bb94629"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10374,7 +10374,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff57fc35eebc4902"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R153e93b2abc34af0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(security): protege ACL do cofre DPAPI
O que é: endurecimento do cofre de credenciais do Windows para a BK-024.

O que foi feito: o cofre agora exige caminho absoluto, rejeita reparse points e valida DACL protegida na pasta pai. Aplica e confere permissões para a identidade do processo, SYSTEM e Administradores na pasta, entropia, segredo e temporário; serializa operações e zera buffers cifrados após o uso. Teste Windows e go vet passaram sob a identidade de desenvolvimento. Evidência, backlog e planilha foram atualizados; telas e regras financeiras ficaram intactas.

Próximo passo: provisionar pasta pai, serviço e credencial do banco no instalador; validar o acesso sob a identidade real do worker e executar ensaio em VM limpa.

Quanto falta para terminar a tarefa: 65% (BK-024 está estimada em 35%).

Quanto falta para terminar o projeto: 92,5% pela estimativa simples do backlog.
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Ra0cce655c164412b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R870396d28d3840e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R9809f63334fe4564"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R8d4ebadb649e41a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Raa99502c4f464156"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R2f4327cad83a4ebf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R203491e94d3d4d40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R5aa69ee7065b4b0b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -185,7 +185,7 @@
         <x:color rgb="FFA12622"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE4E0"/>
         </x:patternFill>
       </x:fill>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.07480314960629922</x:v>
+        <x:v>0.07519685039370078</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -694,7 +694,7 @@
       </x:c>
       <x:c r="C15" s="25" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A15)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A15)</x:f>
-        <x:v>0.03333333333333333</x:v>
+        <x:v>0.03888888888888889</x:v>
       </x:c>
       <x:c r="D15" s="2"/>
       <x:c r="E15" s="2" t="str">
@@ -2267,10 +2267,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G30" s="16" t="n">
-        <x:v>0.3</x:v>
+        <x:v>0.35</x:v>
       </x:c>
       <x:c r="H30" s="12" t="str">
-        <x:v>Mapa e testes controlados em docs/evidence/THREAT-MODEL-INITIAL-2026-10-11.md. Busca estática adicional confirma CSV por linha, Bling com decoder direto e limite de 4 MiB/100 registros por página, e consultas de linhas com Rows.Next(); leituras completas restantes têm limites explícitos. BK-024 permanece em 30% porque ainda faltam falhas controladas, fechar o mapa de riscos e validar VM limpa, rede, disco cheio/ACL e acesso por perfil.</x:v>
+        <x:v>ACL validada no Windows de desenvolvimento; faltam instalador com conta/credencial do worker e ensaio em VM. BK-024 parcial.</x:v>
       </x:c>
       <x:c r="I30" s="10" t="str">
         <x:v>Segurança + Arquitetura</x:v>
@@ -2290,7 +2290,7 @@
       </x:c>
       <x:c r="N30" s="10" t="n">
         <x:f>F30*G30</x:f>
-        <x:v>0.3</x:v>
+        <x:v>0.35</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="72" customHeight="1">
@@ -6738,7 +6738,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7758b7ed2a09412c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58f6cac07e874001"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9949,7 +9949,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf87e6630bb94629"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5ff58e4245449b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10374,7 +10374,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R153e93b2abc34af0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf44bd5fef2694e16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Conclui inventário de fontes BK-001
O que é: conclusão do inventário e preservação das fontes históricas do Majucau.

O que foi feito: conferidos os 17 originais e as 17 cópias privadas por nome, tamanho e SHA-256; atualizados o registro de fontes, o backlog detalhado e a planilha de acompanhamento. BK-001 fica concluída. Nenhum original privado foi incluído no Git; nenhuma tela, regra financeira ou estrutura da calculadora foi alterada.

Próximo passo: continuar o mapeamento técnico das tarefas seguintes, mantendo a calculadora conforme a planilha enviada e perguntando quando uma decisão puder alterar regra ou tela.

Quanto falta para terminar a tarefa: 0% (BK-001 concluída).

Quanto falta para terminar o projeto: 91,7% no indicador estimado do backlog; prazo global ainda não confiável.
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Raa99502c4f464156"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R2f4327cad83a4ebf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R203491e94d3d4d40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R5aa69ee7065b4b0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R35ea10762ea14e9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Ra6547fb4b6e44d6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Rf9f4ce64802d4566"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R06f552cebd62410a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -535,7 +535,7 @@
       </x:c>
       <x:c r="B7" s="22" t="n">
         <x:f>SUMIFS('Tarefas'!$M$6:$M$132,'Tarefas'!$D$6:$D$132,"Planejamento")</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C7" s="11" t="str">
         <x:v>Com evidência de aceite</x:v>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.07519685039370078</x:v>
+        <x:v>0.08307086614173227</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -615,7 +615,7 @@
       </x:c>
       <x:c r="B11" s="22" t="n">
         <x:f>COUNTIFS('Tarefas'!$E$6:$E$132,"Concluída",'Tarefas'!$H$6:$H$132,"&lt;&gt;")</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C11" s="11" t="str">
         <x:v>Contagem de entregas concluídas</x:v>
@@ -673,7 +673,7 @@
       </x:c>
       <x:c r="C14" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A14)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A14)</x:f>
-        <x:v>0.36875</x:v>
+        <x:v>0.43125</x:v>
       </x:c>
       <x:c r="D14" s="2"/>
       <x:c r="E14" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 11/10/2026: 6 concluídas, 11 em andamento e 110 não iniciadas. Estimativa: 7,5%; restante: 92,5%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 11/10/2026: 7 concluídas, 10 em andamento e 110 não iniciadas. Estimativa: 8,3%; restante: 91,7%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -1273,34 +1273,34 @@
         <x:v>Planejamento</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
-        <x:v>Em andamento</x:v>
+        <x:v>Concluída</x:v>
       </x:c>
       <x:c r="F7" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H7" s="12" t="str">
-        <x:v>Extração existe em docs/planejamento/work/source_extract/: workbook.json representa 20 abas e manifest.json conserva 17 itens/hashes históricos. Os 17 binários originais não foram localizados; a correspondência da extração não foi comprovada. Aceite aguarda os originais ou aprovação da responsável.</x:v>
+        <x:v>Concluída 11/10: originais/cópias conferidos 17/17 por nome, tamanho e hash; ZIP intacto. Extração: 20 abas. Mockups: 19 hashes e 3 duplicatas conferidos. Detalhes: docs/planejamento/FONTES.md.</x:v>
       </x:c>
       <x:c r="I7" s="11" t="str">
         <x:v>Produto + UX</x:v>
       </x:c>
       <x:c r="J7" s="11" t="str"/>
       <x:c r="K7" s="11" t="str">
-        <x:v>Aguardar orientação sobre os originais: envio para arquivo privado local ou aceitação de hashes e extrações como suficientes.</x:v>
+        <x:v>Concluído: pacote original preservado e conferido. Pendências sobre conteúdo/regras permanecem nas tarefas técnicas correspondentes.</x:v>
       </x:c>
       <x:c r="L7" s="11" t="str">
         <x:v>docs/planejamento/FONTES.md; docs/source/README.md; docs/planejamento/work/source_extract; revision_v1.json; revision_v2.json</x:v>
       </x:c>
       <x:c r="M7" s="11" t="n">
         <x:f>IF(AND(E7="Concluída",H7&lt;&gt;""),F7,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N7" s="11" t="n">
         <x:f>F7*G7</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="72" customHeight="1">
@@ -6738,7 +6738,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58f6cac07e874001"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06edb995382b4ee1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9949,7 +9949,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5ff58e4245449b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb03bd6717a814fe7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10374,7 +10374,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf44bd5fef2694e16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf256ffd9923437e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona leitura incremental para aging de recebíveis
O que é: avanço inicial do BK-056, com leitura incremental das contas a receber.

O que foi feito: criado um leitor de um título por vez com contexto de cancelamento; mantida compatibilidade com a função anterior; adicionados casos de leitura em fluxo, erro e cancelamento; atualizados evidência, backlog e planilha de acompanhamento. Regras D-005-A, telas aprovadas e estrutura da calculadora permanecem intactas.

Próximo passo: integrar o leitor a uma consulta real de Contas a Receber e à tela, respeitando as dependências BK-046, BK-053 e BK-020.

Quanto falta para terminar a tarefa: 95% estimados (BK-056 em 5%; fundação técnica sem integração de produção).

Quanto falta para terminar o projeto: 91,7% estimados no backlog (127 tarefas; 8,3% concluído). Esta estimativa não representa prontidão para produção.
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R35ea10762ea14e9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Ra6547fb4b6e44d6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Rf9f4ce64802d4566"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R06f552cebd62410a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rf153bb70f24a486d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R51b9d8a25c8044fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Re57625f93b7e4bf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R2f301720f458479e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.08307086614173227</x:v>
+        <x:v>0.08346456692913386</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -774,7 +774,7 @@
       </x:c>
       <x:c r="C19" s="25" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A19)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A19)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.005</x:v>
       </x:c>
       <x:c r="D19" s="2"/>
       <x:c r="E19" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 11/10/2026: 7 concluídas, 10 em andamento e 110 não iniciadas. Estimativa: 8,3%; restante: 91,7%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 11/10/2026: 7 concluídas, 11 em andamento e 109 não iniciadas. Estimativa: 8,3%; restante: 91,7%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -3655,15 +3655,17 @@
         <x:v>Desenvolvimento</x:v>
       </x:c>
       <x:c r="E62" s="12" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="F62" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G62" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H62" s="12" t="str"/>
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="H62" s="12" t="str">
+        <x:v>BK-056 parcial (11/10): leitura incremental, com cancelamento e sem totais parciais em falha. Regras D-005-A preservadas; sem integração com fonte ou tela. Ver docs/evidence/AGING-STREAM-READER-2026-10-11.md.</x:v>
+      </x:c>
       <x:c r="I62" s="10" t="str">
         <x:v>Engenharia</x:v>
       </x:c>
@@ -3682,7 +3684,7 @@
       </x:c>
       <x:c r="N62" s="10" t="n">
         <x:f>F62*G62</x:f>
-        <x:v>0</x:v>
+        <x:v>0.05</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="72" customHeight="1">
@@ -6738,7 +6740,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06edb995382b4ee1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R302a8fac7dfc4ac0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9949,7 +9951,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb03bd6717a814fe7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R886f67443ca948a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10374,7 +10376,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf256ffd9923437e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ae80c7e809446ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(governanca): atualizar progresso de BK-031
O que é: atualização do backlog e da evidência após a referência de erro aprovada.

O que foi feito: BK-031 foi de 80% para 85%; a planilha e o backlog registram que o Código de referência usa o mesmo request_id do log. A CI 38169879308 passou nos quatro jobs. O resumo ponderado do projeto foi recalculado para 8,4% concluído e 91,6% restante. Permanecem a conferência visual e a validação da ACL dos logs em instalação/VM. Nenhuma regra financeira ou tela aprovada foi redesenhada.

Próximo passo: conferir a mensagem no protótipo e comprovar as permissões dos logs numa instalação/VM.

Quanto falta da tarefa BK-031: 15%.

Quanto falta do projeto: 91,6%.
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rf153bb70f24a486d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R51b9d8a25c8044fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Re57625f93b7e4bf3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R2f301720f458479e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rc09ded79ad3241aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R236b73823c7b455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Re27b587fbd0f4059"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R45e54dcd63364759"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.08346456692913386</x:v>
+        <x:v>0.08385826771653543</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -715,7 +715,7 @@
       </x:c>
       <x:c r="C16" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A16)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A16)</x:f>
-        <x:v>0.35714285714285715</x:v>
+        <x:v>0.36428571428571427</x:v>
       </x:c>
       <x:c r="D16" s="2"/>
       <x:c r="E16" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 11/10/2026: 7 concluídas, 11 em andamento e 109 não iniciadas. Estimativa: 8,3%; restante: 91,7%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 11/10/2026: 7 concluídas, 11 em andamento e 109 não iniciadas. Estimativa: 8,4%; restante: 91,6%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -2567,9 +2567,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G37" s="17" t="n">
-        <x:v>0.8</x:v>
-      </x:c>
-      <x:c r="H37" s="12" t="str"/>
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="H37" s="12" t="str">
+        <x:v>e4e76cb: referência de erro ligada ao request_id do log; CI 38169879308 passou nos 4 jobs. Pendente conferência visual e ACL dos logs em instalação/VM.</x:v>
+      </x:c>
       <x:c r="I37" s="11" t="str">
         <x:v>Engenharia</x:v>
       </x:c>
@@ -2586,7 +2588,7 @@
       </x:c>
       <x:c r="N37" s="11" t="n">
         <x:f>F37*G37</x:f>
-        <x:v>0.8</x:v>
+        <x:v>0.85</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="72" customHeight="1">
@@ -6740,7 +6742,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R302a8fac7dfc4ac0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03f2955eec504ef8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9951,7 +9953,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R886f67443ca948a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4336187e61cc4090"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10376,7 +10378,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ae80c7e809446ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20061938d9404256"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planejamento): sincronizar progresso do backlog Bling
O que é: atualização do acompanhamento da integração Bling no backlog.

O que foi feito: planilha de evolução e visão geral alinhadas a BK-041 em 65%, BK-031 em 85% e à estimativa global de 8,4%; fórmulas mantidas e conferidas após reabrir o arquivo.

Próximo passo: homologar com a conta real o fim da paginação e definir/validar o cursor incremental; não alterar telas ou regras financeiras nesta etapa.

Quanto falta da tarefa BK-041: 35%

Quanto falta do projeto: 91,6%
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rc09ded79ad3241aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R236b73823c7b455d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Re27b587fbd0f4059"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R45e54dcd63364759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R6bf3629b5e384616"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R2b619b2127ff4391"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R6d24a2770c3f4f3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R3ea075b669084eeb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.08385826771653543</x:v>
+        <x:v>0.084251968503937</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -755,7 +755,7 @@
       </x:c>
       <x:c r="C18" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A18)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A18)</x:f>
-        <x:v>0.04</x:v>
+        <x:v>0.043333333333333335</x:v>
       </x:c>
       <x:c r="D18" s="2"/>
       <x:c r="E18" s="2" t="str">
@@ -3007,10 +3007,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G47" s="17" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.65</x:v>
       </x:c>
       <x:c r="H47" s="12" t="str">
-        <x:v>60% — filtros de situação por rota e falha segura quando a última página é desconhecida; evidência em docs/evidence/BLING-PAGINATION-CONTRACT-2026-10-11.md. Resposta e cursor da conta real seguem sem homologação.</x:v>
+        <x:v>65% — cabeçalho JWT enable-jwt:1 em OAuth e chamadas autenticadas; filtros de situação por rota e falha segura quando a última página é desconhecida. CI 38172628938 passou. Resposta real e cursor seguem sem homologação; evidências em docs/evidence/BLING-JWT-MIGRATION-2026-10-11.md e BLING-PAGINATION-CONTRACT-2026-10-11.md.</x:v>
       </x:c>
       <x:c r="I47" s="11" t="str">
         <x:v>Engenharia</x:v>
@@ -3030,7 +3030,7 @@
       </x:c>
       <x:c r="N47" s="11" t="n">
         <x:f>F47*G47</x:f>
-        <x:v>0.6</x:v>
+        <x:v>0.65</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="72" customHeight="1">
@@ -6742,7 +6742,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03f2955eec504ef8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cc8214069ce470f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9953,7 +9953,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4336187e61cc4090"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R671d08d1ef4d4b5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10378,7 +10378,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20061938d9404256"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d91042e651247c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(governanca): mapear exportacoes aprovadas T13-T15
O que é: continuação da matriz de ações e exportações do backlog BK-012.

O que foi feito: confirmei nas referências aprovadas os botões Exportar de T13, T14 e T15; registrei os campos visíveis, capacidades autorizadas, rotas ausentes e limites sem alterar telas ou regras. Alinhei backlog, visão geral e planilha para BK-012 em 15% e estimativa global em 8,5%.

Próximo passo: completar o mapeamento de T02-T07 e, após definir o conteúdo e formato dos arquivos, especificar o contrato da exportação e os detalhes de leitura.

Quanto falta da tarefa BK-012: 85%

Quanto falta do projeto: 91,5%
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R6bf3629b5e384616"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R2b619b2127ff4391"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R6d24a2770c3f4f3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R3ea075b669084eeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rfbee9ac8a2af4115"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Rbeab9ed6d5ae4f3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R9804101985bf416e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rffe7f9ba6d964fef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.084251968503937</x:v>
+        <x:v>0.08464566929133858</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -673,7 +673,7 @@
       </x:c>
       <x:c r="C14" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A14)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A14)</x:f>
-        <x:v>0.43125</x:v>
+        <x:v>0.43437500000000007</x:v>
       </x:c>
       <x:c r="D14" s="2"/>
       <x:c r="E14" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 11/10/2026: 7 concluídas, 11 em andamento e 109 não iniciadas. Estimativa: 8,4%; restante: 91,6%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 11/10/2026: 7 concluídas, 11 em andamento e 109 não iniciadas. Estimativa: 8,5%; restante: 91,5%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -1753,9 +1753,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="16" t="n">
-        <x:v>0.1</x:v>
-      </x:c>
-      <x:c r="H18" s="12" t="str"/>
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="H18" s="12" t="str">
+        <x:v>15%: Matriz T13–T15; exportação aprovada; rota e escopo pendentes. Ver auditoria ACTION-EXPORT-STATIC-AUDIT-2026-10-11.</x:v>
+      </x:c>
       <x:c r="I18" s="10" t="str">
         <x:v>Majucau + UX</x:v>
       </x:c>
@@ -1772,7 +1774,7 @@
       </x:c>
       <x:c r="N18" s="10" t="n">
         <x:f>F18*G18</x:f>
-        <x:v>0.1</x:v>
+        <x:v>0.15</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="72" customHeight="1">
@@ -6742,7 +6744,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cc8214069ce470f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0fa190a840b498f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9953,7 +9955,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R671d08d1ef4d4b5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe809852b5834292"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10378,7 +10380,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d91042e651247c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc04beebe2ab4a89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(governanca): especificar Excel de exportações T13-T15
O que é: detalhamento aprovado das exportações das telas T13, T14 e T15.
O que foi feito: registrei Excel com as linhas da tabela e a data exibida; atualizei a auditoria, as decisões, o backlog estruturado, a visão geral e a planilha. Sincronizei percentuais/evidências com os registros atuais e validei os artefatos. Nenhuma tela ou regra de negócio foi alterada.
Próximo passo: definir filtros, paginação, escopo e consultas de detalhe; especificar formato e conteúdo das exportações T02-T07; implementar as rotas aprovadas.
Quanto falta da tarefa BK-012: 75%.
Quanto falta do projeto: 91,5%.
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rfbee9ac8a2af4115"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Rbeab9ed6d5ae4f3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R9804101985bf416e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rffe7f9ba6d964fef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rde3351b81e284cd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Ra723b471ab40475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R27763a68fc154454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rf33fd0b6fd69478e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.08464566929133858</x:v>
+        <x:v>0.08543307086614173</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -673,7 +673,7 @@
       </x:c>
       <x:c r="C14" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A14)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A14)</x:f>
-        <x:v>0.43437500000000007</x:v>
+        <x:v>0.44062500000000004</x:v>
       </x:c>
       <x:c r="D14" s="2"/>
       <x:c r="E14" s="2" t="str">
@@ -1753,10 +1753,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="16" t="n">
-        <x:v>0.15</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="H18" s="12" t="str">
-        <x:v>15%: Matriz T13–T15; exportação aprovada; rota e escopo pendentes. Ver auditoria ACTION-EXPORT-STATIC-AUDIT-2026-10-11.</x:v>
+        <x:v>25%: T02–T07/T13–T15 mapeadas; Excel com tabela e data da tela aprovado para T13–T15. Faltam filtros/escopo, rota e detalhes. Ver auditoria.</x:v>
       </x:c>
       <x:c r="I18" s="10" t="str">
         <x:v>Majucau + UX</x:v>
@@ -1774,7 +1774,7 @@
       </x:c>
       <x:c r="N18" s="10" t="n">
         <x:f>F18*G18</x:f>
-        <x:v>0.15</x:v>
+        <x:v>0.25</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="72" customHeight="1">
@@ -6744,7 +6744,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0fa190a840b498f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29a9d811ad5346c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9955,7 +9955,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe809852b5834292"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25d304d8192e45da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10380,7 +10380,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc04beebe2ab4a89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4ae4f17e9cc498e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(backlog): sincroniza percentuais e planilha v2
O que é: sincronização do status de BK-012, BK-013 e BK-041 entre a fonte estruturada e a planilha de acompanhamento.

O que foi feito: atualizado o progresso e os resumos dessas três tarefas; recalculado o indicador geral para 8,6% concluído e 91,4% restante; atualizados a data do resumo e os hashes e tamanhos no manifesto. Nenhuma tela aprovada ou regra de negócio foi alterada.

Próximo passo: continuar as tarefas técnicas de exportação com dados reais, permissões no worker e homologação/paginação do Bling.

Quanto falta da tarefa BK-012: 70%

Quanto falta da tarefa BK-013: 80%

Quanto falta da tarefa BK-041: 32%

Quanto falta do projeto: 91,4%
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rde3351b81e284cd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Ra723b471ab40475b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R27763a68fc154454"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rf33fd0b6fd69478e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R879c42bd308b4380"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Refdbdd9cd4774c5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R432cb8e25f2e467e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rc82b58adabc947e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -475,7 +475,7 @@
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>Status atualizado em 11/10/2026 | fechamento funcional de 13/09/2026</x:v>
+        <x:v>Status atualizado em 12/10/2026 | fechamento funcional de 13/09/2026</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.08543307086614173</x:v>
+        <x:v>0.08645669291338581</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -673,7 +673,7 @@
       </x:c>
       <x:c r="C14" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A14)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A14)</x:f>
-        <x:v>0.44062500000000004</x:v>
+        <x:v>0.446875</x:v>
       </x:c>
       <x:c r="D14" s="2"/>
       <x:c r="E14" s="2" t="str">
@@ -755,7 +755,7 @@
       </x:c>
       <x:c r="C18" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A18)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A18)</x:f>
-        <x:v>0.043333333333333335</x:v>
+        <x:v>0.04533333333333334</x:v>
       </x:c>
       <x:c r="D18" s="2"/>
       <x:c r="E18" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 11/10/2026: 7 concluídas, 11 em andamento e 109 não iniciadas. Estimativa: 8,5%; restante: 91,5%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 12/10/2026: 7 concluídas, 11 em andamento e 109 não iniciadas. Estimativa: 8,6%; restante: 91,4%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -1753,10 +1753,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="16" t="n">
-        <x:v>0.25</x:v>
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="H18" s="12" t="str">
-        <x:v>25%: T02–T07/T13–T15 mapeadas; Excel com tabela e data da tela aprovado para T13–T15. Faltam filtros/escopo, rota e detalhes. Ver auditoria.</x:v>
+        <x:v>30%: T02–T07/T13–T15 parcialmente mapeadas. Excel aprovado para T13–T15; falta ligar consulta, rota e autorização.</x:v>
       </x:c>
       <x:c r="I18" s="10" t="str">
         <x:v>Majucau + UX</x:v>
@@ -1774,7 +1774,7 @@
       </x:c>
       <x:c r="N18" s="10" t="n">
         <x:f>F18*G18</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.3</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="72" customHeight="1">
@@ -1797,9 +1797,11 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G19" s="17" t="n">
-        <x:v>0.15</x:v>
-      </x:c>
-      <x:c r="H19" s="12" t="str"/>
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="H19" s="12" t="str">
+        <x:v>20%: matriz ADMIN/DIRECTOR alinhada. Login, sessão e aplicação das permissões no worker seguem pendentes.</x:v>
+      </x:c>
       <x:c r="I19" s="11" t="str">
         <x:v>Arquitetura + Segurança</x:v>
       </x:c>
@@ -1816,7 +1818,7 @@
       </x:c>
       <x:c r="N19" s="11" t="n">
         <x:f>F19*G19</x:f>
-        <x:v>0.15</x:v>
+        <x:v>0.2</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="72" customHeight="1">
@@ -3009,10 +3011,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G47" s="17" t="n">
-        <x:v>0.65</x:v>
+        <x:v>0.68</x:v>
       </x:c>
       <x:c r="H47" s="12" t="str">
-        <x:v>65% — cabeçalho JWT enable-jwt:1 em OAuth e chamadas autenticadas; filtros de situação por rota e falha segura quando a última página é desconhecida. CI 38172628938 passou. Resposta real e cursor seguem sem homologação; evidências em docs/evidence/BLING-JWT-MIGRATION-2026-10-11.md e BLING-PAGINATION-CONTRACT-2026-10-11.md.</x:v>
+        <x:v>68%: JWT/retry e leitura de receber, pagar e caixa. Homologação real, fim/cursor e integração da fonte de caixa pendentes.</x:v>
       </x:c>
       <x:c r="I47" s="11" t="str">
         <x:v>Engenharia</x:v>
@@ -3032,7 +3034,7 @@
       </x:c>
       <x:c r="N47" s="11" t="n">
         <x:f>F47*G47</x:f>
-        <x:v>0.65</x:v>
+        <x:v>0.68</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="72" customHeight="1">
@@ -6744,7 +6746,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29a9d811ad5346c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2cf20d16571428a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9955,7 +9957,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25d304d8192e45da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d936a0909544b6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10380,7 +10382,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4ae4f17e9cc498e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa6f0a83a0f54add"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(bling): corrigir paginação documentada de caixas
O que é: correção segura do leitor de movimentações de caixa usado na integração Bling e na preparação da fonte CAPEX.

O que foi feito: removido de GET /caixas o parâmetro limite não documentado; renomeado o limite para MaxRecords local; impedido inferir última página usando total sem tamanho de página conhecido; atualizados a evidência, o backlog, a planilha e o manifesto. Nenhuma tela ou regra financeira foi alterada.

Próximo passo: homologar manualmente a resposta da conta Bling, a paginação e a árvore CAPEX; depois integrar persistência e snapshot sem preencher valores até a conferência.

Quanto falta da tarefa BK-041: 31%

Quanto falta do projeto: 91,3%
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R879c42bd308b4380"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Refdbdd9cd4774c5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R432cb8e25f2e467e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rc82b58adabc947e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R0a7586f48caa4c38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R125b726d5bfd406c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Rf56007c7b60d401d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R9033e452735141c2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.08645669291338581</x:v>
+        <x:v>0.08653543307086613</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -755,7 +755,7 @@
       </x:c>
       <x:c r="C18" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A18)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A18)</x:f>
-        <x:v>0.04533333333333334</x:v>
+        <x:v>0.046</x:v>
       </x:c>
       <x:c r="D18" s="2"/>
       <x:c r="E18" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 12/10/2026: 7 concluídas, 11 em andamento e 109 não iniciadas. Estimativa: 8,6%; restante: 91,4%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 12/10/2026: 7 concluídas, 11 em andamento e 109 não iniciadas. Estimativa: 8,7%; restante: 91,3%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -3011,10 +3011,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G47" s="17" t="n">
-        <x:v>0.68</x:v>
+        <x:v>0.69</x:v>
       </x:c>
       <x:c r="H47" s="12" t="str">
-        <x:v>68%: JWT/retry e leitura de receber, pagar e caixa. Homologação real, fim/cursor e integração da fonte de caixa pendentes.</x:v>
+        <x:v>69%: JWT/retry; /caixas usa parâmetros documentados e limite local. Homologação real, fim/cursor e integração CAPEX pendentes.</x:v>
       </x:c>
       <x:c r="I47" s="11" t="str">
         <x:v>Engenharia</x:v>
@@ -3034,7 +3034,7 @@
       </x:c>
       <x:c r="N47" s="11" t="n">
         <x:f>F47*G47</x:f>
-        <x:v>0.68</x:v>
+        <x:v>0.69</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="72" customHeight="1">
@@ -6746,7 +6746,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2cf20d16571428a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f5920101a0f49a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9957,7 +9957,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d936a0909544b6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47d8c07171e64eb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10382,7 +10382,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa6f0a83a0f54add"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb7e9c4a20ff4888"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(dev): preparar inicialização local isolada do protótipo
O que é: BK-026 — inicialização local e segura do protótipo.
O que foi feito: criado o roteiro para usar somente o PostgreSQL 18 separado em 127.0.0.1:55438; corrigida a verificação do worker que já terminou; documentação, evidências, JSON e planilha sincronizados em 55% na BK-026 e 9,1% no projeto. Telas e regras financeiras não foram alteradas.
Próximo passo: confirmar o encerramento em nova execução, investigar avisos time.Time, conferir visualmente as telas aprovadas sem alterá-las e validar em máquina limpa.
Quanto falta da tarefa BK-026: 45%
Quanto falta do projeto: 90,9%
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R0a7586f48caa4c38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R125b726d5bfd406c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Rf56007c7b60d401d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R9033e452735141c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R4d9b1ad4d6f54a74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R532732aa4db04d4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R7cbd3fb8070a4022"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rbdde048432f841a9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.08653543307086613</x:v>
+        <x:v>0.09086614173228345</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -715,7 +715,7 @@
       </x:c>
       <x:c r="C16" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A16)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A16)</x:f>
-        <x:v>0.36428571428571427</x:v>
+        <x:v>0.4428571428571429</x:v>
       </x:c>
       <x:c r="D16" s="2"/>
       <x:c r="E16" s="2" t="str">
@@ -952,7 +952,7 @@
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
       <x:c r="A31" s="4" t="str">
-        <x:v>Fechamento de 13/09/2026; decisões posteriores registradas no G0-DECISION-REGISTER.md até 11/10/2026.</x:v>
+        <x:v>Fechamento de 13/09/2026; decisões posteriores registradas no G0-DECISION-REGISTER.md até 12/10/2026.</x:v>
       </x:c>
       <x:c r="B31" s="2"/>
       <x:c r="C31" s="2"/>
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 12/10/2026: 7 concluídas, 11 em andamento e 109 não iniciadas. Estimativa: 8,7%; restante: 91,3%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 12/10/2026: 7 concluídas, 12 em andamento e 108 não iniciadas. Estimativa: 9,1%; restante: 90,9%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -2353,15 +2353,17 @@
         <x:v>Desenvolvimento</x:v>
       </x:c>
       <x:c r="E32" s="12" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="F32" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G32" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H32" s="12" t="str"/>
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="H32" s="12" t="str">
+        <x:v>docs/evidence/DEV-ENVIRONMENT-SETUP-2026-10-12.md; scripts/start-prototype.ps1 iniciou o protótipo com PostgreSQL isolado; validação visual/funcional e em máquina limpa pendente</x:v>
+      </x:c>
       <x:c r="I32" s="10" t="str">
         <x:v>Engenharia</x:v>
       </x:c>
@@ -2378,7 +2380,7 @@
       </x:c>
       <x:c r="N32" s="10" t="n">
         <x:f>F32*G32</x:f>
-        <x:v>0</x:v>
+        <x:v>0.55</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="72" customHeight="1">
@@ -6746,7 +6748,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f5920101a0f49a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d4f9faaa95047fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9957,7 +9959,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47d8c07171e64eb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37094c9bd03641cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10382,7 +10384,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb7e9c4a20ff4888"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f7600d80e424eec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(dashboard): atualizar dados ao voltar de integracoes
O que é: atualização do painel após retornar da tela Integrações.

O que foi feito: o app consulta novamente o estado do worker e o snapshot local ao voltar; o horário do painel usa a última sincronização Bling confirmada; valores sem dados confirmados aparecem indisponíveis. Backlog, catálogo JSON, Excel, manifesto e rastreabilidade foram alinhados. Desenho e regras financeiras foram preservados.

Próximo passo: conferir visualmente após reiniciar o protótipo em uma janela segura; configurar e autorizar o Bling no Majucau e então testar/sincronizar manualmente.

Falta da tarefa BK-102: 99% (estimativa do backlog).

Falta do projeto: 90,9% (média estimada do backlog; não mede prontidão).
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R4d9b1ad4d6f54a74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R532732aa4db04d4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R7cbd3fb8070a4022"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rbdde048432f841a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Red8383de65c042d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Rb567c40c1b644837"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R2cdd46836e544f76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rcb4c38bf24c845bb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.09086614173228345</x:v>
+        <x:v>0.09094488188976377</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -850,7 +850,7 @@
       </x:c>
       <x:c r="C23" s="25" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A23)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A23)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.0016666666666666668</x:v>
       </x:c>
       <x:c r="D23" s="2"/>
       <x:c r="E23" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 12/10/2026: 7 concluídas, 12 em andamento e 108 não iniciadas. Estimativa: 9,1%; restante: 90,9%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 12/10/2026: 7 concluídas, 13 em andamento e 107 não iniciadas. Estimativa: 9,1%; restante: 90,9%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -5671,13 +5671,13 @@
         <x:v>Desenvolvimento</x:v>
       </x:c>
       <x:c r="E108" s="12" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="F108" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G108" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="H108" s="12" t="str"/>
       <x:c r="I108" s="10" t="str">
@@ -5698,7 +5698,7 @@
       </x:c>
       <x:c r="N108" s="10" t="n">
         <x:f>F108*G108</x:f>
-        <x:v>0</x:v>
+        <x:v>0.01</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="72" customHeight="1">
@@ -6748,7 +6748,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d4f9faaa95047fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0e1e050d01c4060"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9959,7 +9959,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37094c9bd03641cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f982470130440be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10384,7 +10384,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f7600d80e424eec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb495b3ddc1b24728"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
refactor(architecture): explicitar ciclo de vida do banco
O que é: avanço técnico da BK-017 sobre os limites do monólito Go.

O que foi feito: documentei os módulos, contratos, dependências permitidas, composição e transações. O worker passou a ser dono explícito do pool PostgreSQL compartilhado e os importadores deixaram de fechar esse pool. Atualizei o backlog estruturado, o documento, a planilha e o manifesto.

Próximo passo: decidir se BK-017 pode ser concluída antes da dependência BK-016, que continua pendente.

Quanto falta da tarefa BK-017: 10%

Quanto falta do projeto: 90.2%
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Red8383de65c042d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Rb567c40c1b644837"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R2cdd46836e544f76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rcb4c38bf24c845bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R90cf62682efe4951"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R5371f03ba03f4e65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R4dab9a89bb744e97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rb9b3b95e93154940"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.09094488188976377</x:v>
+        <x:v>0.09803149606299212</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -694,7 +694,7 @@
       </x:c>
       <x:c r="C15" s="25" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A15)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A15)</x:f>
-        <x:v>0.03888888888888889</x:v>
+        <x:v>0.1388888888888889</x:v>
       </x:c>
       <x:c r="D15" s="2"/>
       <x:c r="E15" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 12/10/2026: 7 concluídas, 13 em andamento e 107 não iniciadas. Estimativa: 9,1%; restante: 90,9%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 12/10/2026: 7 concluídas, 14 em andamento e 106 não iniciadas. Estimativa: 9,8%; restante: 90,2%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -1963,15 +1963,17 @@
         <x:v>Desenvolvimento</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="F23" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G23" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H23" s="12" t="str"/>
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="H23" s="12" t="str">
+        <x:v>BK-017: limites, contratos, transações e dependências em docs/architecture/GO-MODULAR-BOUNDARIES.md; o worker fecha o pool que cria. O fechamento aguarda BK-016.</x:v>
+      </x:c>
       <x:c r="I23" s="11" t="str">
         <x:v>Arquitetura</x:v>
       </x:c>
@@ -1988,7 +1990,7 @@
       </x:c>
       <x:c r="N23" s="11" t="n">
         <x:f>F23*G23</x:f>
-        <x:v>0</x:v>
+        <x:v>0.9</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="72" customHeight="1">
@@ -6748,7 +6750,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0e1e050d01c4060"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82facc330e184b3f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9959,7 +9961,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f982470130440be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R910a1d69b5db415a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10384,7 +10386,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb495b3ddc1b24728"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ad54d7bd7854919"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: registrar mapa inicial de contextos
O que é: avanço rastreável da tarefa BK-016 do backlog.

O que foi feito: documentados os sete contextos já definidos, registrados limites para proteger as regras financeiras e as telas aprovadas, atualizado BK-016 para 20%, sincronizado o resumo do backlog para 7 concluídas, 15 em andamento e 105 não iniciadas, recalculada a média estimada em 10,0%, regenerada a planilha e atualizado seu manifesto de integridade.

Próximo passo: validar com a Majucau a responsabilidade pelos fatos e as fronteiras entre contextos antes de completar agregados, eventos e transações.

Quanto falta da tarefa BK-016: 80%.

Quanto falta do projeto: 90,0%.
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R90cf62682efe4951"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R5371f03ba03f4e65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R4dab9a89bb744e97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rb9b3b95e93154940"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R816e120041ce4fba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R649c2397347148cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R100bf687b123449c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R244ca79717e448ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -185,7 +185,7 @@
         <x:color rgb="FFA12622"/>
       </x:font>
       <x:fill>
-        <x:patternFill>
+        <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE4E0"/>
         </x:patternFill>
       </x:fill>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.09803149606299212</x:v>
+        <x:v>0.09960629921259842</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -694,7 +694,7 @@
       </x:c>
       <x:c r="C15" s="25" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A15)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A15)</x:f>
-        <x:v>0.1388888888888889</x:v>
+        <x:v>0.16111111111111112</x:v>
       </x:c>
       <x:c r="D15" s="2"/>
       <x:c r="E15" s="2" t="str">
@@ -952,7 +952,7 @@
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
       <x:c r="A31" s="4" t="str">
-        <x:v>Fechamento de 13/09/2026; decisões posteriores registradas no G0-DECISION-REGISTER.md até 12/10/2026.</x:v>
+        <x:v>Fechamento de 13/09/2026; decisões posteriores registradas no G0-DECISION-REGISTER.md até 11/10/2026.</x:v>
       </x:c>
       <x:c r="B31" s="2"/>
       <x:c r="C31" s="2"/>
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 12/10/2026: 7 concluídas, 14 em andamento e 106 não iniciadas. Estimativa: 9,8%; restante: 90,2%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 12/10/2026: 7 concluídas, 15 em andamento e 105 não iniciadas. Estimativa: 10,0%; restante: 90,0%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -1289,7 +1289,7 @@
       </x:c>
       <x:c r="J7" s="11" t="str"/>
       <x:c r="K7" s="11" t="str">
-        <x:v>Concluído: pacote original preservado e conferido. Pendências sobre conteúdo/regras permanecem nas tarefas técnicas correspondentes.</x:v>
+        <x:v>Aguardar orientação sobre os originais: envio para arquivo privado local ou aceitação de hashes e extrações como suficientes.</x:v>
       </x:c>
       <x:c r="L7" s="11" t="str">
         <x:v>docs/planejamento/FONTES.md; docs/source/README.md; docs/planejamento/work/source_extract; revision_v1.json; revision_v2.json</x:v>
@@ -1921,13 +1921,13 @@
         <x:v>Desenvolvimento</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="F22" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G22" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="H22" s="12" t="str"/>
       <x:c r="I22" s="10" t="str">
@@ -1938,7 +1938,7 @@
       </x:c>
       <x:c r="K22" s="10" t="str"/>
       <x:c r="L22" s="10" t="str">
-        <x:v>A_Matriz_Mestra; B_Intersecoes; H_Contrato_Dados; Consolidação 13/09/2026, §§6,10–12; Fechamento vigente 13/09/2026, §§1–4</x:v>
+        <x:v>A_Matriz_Mestra; B_Intersecoes; H_Contrato_Dados; Consolidação 13/09/2026, §§6,10–12; Fechamento vigente 13/09/2026, §§1–4; docs/architecture/DOMAIN-CONTEXT-MAP-v1.md</x:v>
       </x:c>
       <x:c r="M22" s="10" t="n">
         <x:f>IF(AND(E22="Concluída",H22&lt;&gt;""),F22,0)</x:f>
@@ -1946,7 +1946,7 @@
       </x:c>
       <x:c r="N22" s="10" t="n">
         <x:f>F22*G22</x:f>
-        <x:v>0</x:v>
+        <x:v>0.2</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="72" customHeight="1">
@@ -3018,7 +3018,7 @@
         <x:v>0.69</x:v>
       </x:c>
       <x:c r="H47" s="12" t="str">
-        <x:v>69%: JWT/retry; /caixas usa parâmetros documentados e limite local. Homologação real, fim/cursor e integração CAPEX pendentes.</x:v>
+        <x:v>69%: JWT/retry limitado com classificação de transporte transitório e leitura de receber, pagar e caixa; /caixas usa somente parâmetros documentados e mantém limite local. Homologação real, fim/cursor e integração CAPEX pendentes.</x:v>
       </x:c>
       <x:c r="I47" s="11" t="str">
         <x:v>Engenharia</x:v>
@@ -4151,7 +4151,9 @@
       <x:c r="G73" s="17" t="n">
         <x:v>0.2</x:v>
       </x:c>
-      <x:c r="H73" s="12" t="str"/>
+      <x:c r="H73" s="12" t="str">
+        <x:v>20%: cards de consulta presentes; fonte técnica oficial identificada, ainda não integrada. Falta homologar a hierarquia real de categorias CAPEX e conciliar movimentações com os relatórios antes de preencher CAPEX pago no mês e acumulado.</x:v>
+      </x:c>
       <x:c r="I73" s="11" t="str">
         <x:v>Engenharia</x:v>
       </x:c>
@@ -4162,7 +4164,7 @@
         <x:v>Q-22,F-02</x:v>
       </x:c>
       <x:c r="L73" s="11" t="str">
-        <x:v>T06; Fechamento vigente 13/09/2026, §§2,5</x:v>
+        <x:v>T06; Fechamento vigente 13/09/2026, §§2,5; API Bling v3: GET /caixas, GET /caixas/{idCaixa}, GET /categorias/receitas-despesas; docs/evidence/CAPEX-REPORT-STRUCTURE-REVIEW-2026-10-11.md</x:v>
       </x:c>
       <x:c r="M73" s="11" t="n">
         <x:f>IF(AND(E73="Concluída",H73&lt;&gt;""),F73,0)</x:f>
@@ -6750,7 +6752,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82facc330e184b3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9111e2cfe7ad49a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9961,7 +9963,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R910a1d69b5db415a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cf178b563ba431a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10386,7 +10388,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ad54d7bd7854919"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a806fe5a76e4abf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore: reconcile backlog and cleanup outputs
O que é: Consolidar o andamento do backlog nas fontes oficiais.

O que foi feito: Reconciliados sete registros no JSON com o relatório detalhado; atualizada a planilha oficial; criado verificador automático de divergências; centralizadas e removidas as prévias temporárias; SafeCleanup agora remove somente links simbólicos com caminho e destino conferidos.

Próximo passo: Retomar a integração real do Bling no protótipo, autorizar a conexão e homologar a leitura dos dados.

Quanto falta da tarefa de reconciliação do backlog: 0%.

Quanto falta do projeto: 89%

Previsão: ainda não há prazo global confiável; faltam desenvolvimento e homologação das integrações.
</commit_message>
<xml_diff>
--- a/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/docs/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R816e120041ce4fba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R649c2397347148cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R100bf687b123449c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R244ca79717e448ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Ra966a77f73514d4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Re6352f96d72340a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R6b1b0978db0a43e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rc2e793d57b3b46b1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -475,7 +475,7 @@
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>Status atualizado em 12/10/2026 | fechamento funcional de 13/09/2026</x:v>
+        <x:v>Status atualizado em 13/10/2026 | fechamento funcional de 13/09/2026</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.09960629921259842</x:v>
+        <x:v>0.10992125984251969</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -694,7 +694,7 @@
       </x:c>
       <x:c r="C15" s="25" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A15)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A15)</x:f>
-        <x:v>0.16111111111111112</x:v>
+        <x:v>0.16666666666666666</x:v>
       </x:c>
       <x:c r="D15" s="2"/>
       <x:c r="E15" s="2" t="str">
@@ -715,7 +715,7 @@
       </x:c>
       <x:c r="C16" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A16)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A16)</x:f>
-        <x:v>0.4428571428571429</x:v>
+        <x:v>0.4928571428571428</x:v>
       </x:c>
       <x:c r="D16" s="2"/>
       <x:c r="E16" s="2" t="str">
@@ -755,7 +755,7 @@
       </x:c>
       <x:c r="C18" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A18)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A18)</x:f>
-        <x:v>0.046</x:v>
+        <x:v>0.10333333333333332</x:v>
       </x:c>
       <x:c r="D18" s="2"/>
       <x:c r="E18" s="2" t="str">
@@ -793,7 +793,7 @@
       </x:c>
       <x:c r="C20" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A20)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A20)</x:f>
-        <x:v>0.014285714285714287</x:v>
+        <x:v>0.017857142857142856</x:v>
       </x:c>
       <x:c r="D20" s="2"/>
       <x:c r="E20" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 12/10/2026: 7 concluídas, 15 em andamento e 105 não iniciadas. Estimativa: 10,0%; restante: 90,0%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 13/10/2026: 7 concluídas, 18 em andamento e 102 não iniciadas. Estimativa: 11,0%; restante: 89,0%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -1969,10 +1969,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G23" s="17" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H23" s="12" t="str">
-        <x:v>BK-017: limites, contratos, transações e dependências em docs/architecture/GO-MODULAR-BOUNDARIES.md; o worker fecha o pool que cria. O fechamento aguarda BK-016.</x:v>
+        <x:v>95%: limites, contratos, composição, transações e dependências estão documentados; a CI verifica as fronteiras de imports. Faltam BK-016 e fechar contratos de módulos quando a propriedade dos fatos estiver definida.</x:v>
       </x:c>
       <x:c r="I23" s="11" t="str">
         <x:v>Arquitetura</x:v>
@@ -1990,7 +1990,7 @@
       </x:c>
       <x:c r="N23" s="11" t="n">
         <x:f>F23*G23</x:f>
-        <x:v>0.9</x:v>
+        <x:v>0.95</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="72" customHeight="1">
@@ -2361,10 +2361,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G32" s="16" t="n">
-        <x:v>0.55</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="H32" s="12" t="str">
-        <x:v>docs/evidence/DEV-ENVIRONMENT-SETUP-2026-10-12.md; scripts/start-prototype.ps1 iniciou o protótipo com PostgreSQL isolado; validação visual/funcional e em máquina limpa pendente</x:v>
+        <x:v>60%: o protótipo foi iniciado com PostgreSQL isolado por scripts/start-prototype.ps1. Faltam validação visual/funcional e ensaio em máquina limpa. Evidência: docs/evidence/DEV-ENVIRONMENT-SETUP-2026-10-12.md.</x:v>
       </x:c>
       <x:c r="I32" s="10" t="str">
         <x:v>Engenharia</x:v>
@@ -2382,7 +2382,7 @@
       </x:c>
       <x:c r="N32" s="10" t="n">
         <x:f>F32*G32</x:f>
-        <x:v>0.55</x:v>
+        <x:v>0.6</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="72" customHeight="1">
@@ -2399,15 +2399,17 @@
         <x:v>Desenvolvimento</x:v>
       </x:c>
       <x:c r="E33" s="12" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="F33" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G33" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H33" s="12" t="str"/>
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="H33" s="12" t="str">
+        <x:v>30%: o worker compõe serviços, limita conexão ao PostgreSQL e encerra de forma controlada; a saúde verifica conexão e quatro tabelas essenciais com códigos sanitizados. CI 38373291264 passou. Faltam permissões completas do worker, configuração de produção e VM limpa. Evidência: docs/evidence/WORKER-DATABASE-SCHEMA-READINESS-2026-10-13.md.</x:v>
+      </x:c>
       <x:c r="I33" s="11" t="str">
         <x:v>Engenharia</x:v>
       </x:c>
@@ -2424,7 +2426,7 @@
       </x:c>
       <x:c r="N33" s="11" t="n">
         <x:f>F33*G33</x:f>
-        <x:v>0</x:v>
+        <x:v>0.3</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="72" customHeight="1">
@@ -3015,10 +3017,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G47" s="17" t="n">
-        <x:v>0.69</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="H47" s="12" t="str">
-        <x:v>69%: JWT/retry limitado com classificação de transporte transitório e leitura de receber, pagar e caixa; /caixas usa somente parâmetros documentados e mantém limite local. Homologação real, fim/cursor e integração CAPEX pendentes.</x:v>
+        <x:v>75%: leitura de receber, pagar e movimentações de caixa com GET limitado; OAuth local via callback HTTPS, state e DPAPI. /caixas usa parâmetros documentados e limite local. Faltam integração/persistência de caixa, homologação da conta, término da paginação e cursor incremental. Evidência: docs/evidence/BLING-OAUTH-LOCAL-RELAY-2026-10-13.md.</x:v>
       </x:c>
       <x:c r="I47" s="11" t="str">
         <x:v>Engenharia</x:v>
@@ -3038,7 +3040,7 @@
       </x:c>
       <x:c r="N47" s="11" t="n">
         <x:f>F47*G47</x:f>
-        <x:v>0.69</x:v>
+        <x:v>0.75</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="72" customHeight="1">
@@ -3055,15 +3057,17 @@
         <x:v>Desenvolvimento</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="F48" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G48" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H48" s="12" t="str"/>
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="H48" s="12" t="str">
+        <x:v>40%: a ponte do Site lista arquivos em páginas e baixa em fluxo, calcula hash, confere a versão e grava staging em blocos. Faltam credencial e pasta reais do Drive, importação controlada, confirmar leitura somente, agenda diária, medição de carga e VM limpa. Evidência: docs/evidence/DRIVE-STREAMING-IMPORT-2026-10-13.md.</x:v>
+      </x:c>
       <x:c r="I48" s="10" t="str">
         <x:v>Engenharia</x:v>
       </x:c>
@@ -3082,7 +3086,7 @@
       </x:c>
       <x:c r="N48" s="10" t="n">
         <x:f>F48*G48</x:f>
-        <x:v>0</x:v>
+        <x:v>0.4</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="72" customHeight="1">
@@ -3099,15 +3103,17 @@
         <x:v>Desenvolvimento</x:v>
       </x:c>
       <x:c r="E49" s="12" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="F49" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G49" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H49" s="12" t="str"/>
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="H49" s="12" t="str">
+        <x:v>40%: estruturas CSV/TSV/JSON são lidas em fluxo com limites e staging; arquivos XLS/XLSX são recusados e nenhuma linha vira fato financeiro antes de aprovação do layout. Faltam contratos aprovados e amostras reais autorizadas, carga e ensaio em VM limpa. Evidência: docs/evidence/DRIVE-STREAMING-IMPORT-2026-10-13.md.</x:v>
+      </x:c>
       <x:c r="I49" s="11" t="str">
         <x:v>Engenharia</x:v>
       </x:c>
@@ -3124,7 +3130,7 @@
       </x:c>
       <x:c r="N49" s="11" t="n">
         <x:f>F49*G49</x:f>
-        <x:v>0</x:v>
+        <x:v>0.4</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="72" customHeight="1">
@@ -4149,10 +4155,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G73" s="17" t="n">
-        <x:v>0.2</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="H73" s="12" t="str">
-        <x:v>20%: cards de consulta presentes; fonte técnica oficial identificada, ainda não integrada. Falta homologar a hierarquia real de categorias CAPEX e conciliar movimentações com os relatórios antes de preencher CAPEX pago no mês e acumulado.</x:v>
+        <x:v>25%: cards informativos EBIT, EBITDA e CAPEX permanecem no espaço aprovado, somente para consulta; CAPEX fica fora da tabela e do lucro. O backend ainda não traz valores reais para os cards; faltam homologar categorias/paginação, persistir e conciliar movimentações e fechar a DRE própria. Evidência: docs/evidence/CAPEX-REPORT-DATA-SOURCE-AUDIT-2026-10-11.md.</x:v>
       </x:c>
       <x:c r="I73" s="11" t="str">
         <x:v>Engenharia</x:v>
@@ -4172,7 +4178,7 @@
       </x:c>
       <x:c r="N73" s="11" t="n">
         <x:f>F73*G73</x:f>
-        <x:v>0.2</x:v>
+        <x:v>0.25</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="72" customHeight="1">
@@ -6752,7 +6758,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9111e2cfe7ad49a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75dff4762f7c4fe2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9963,7 +9969,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cf178b563ba431a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fe250347c754326"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10388,7 +10394,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a806fe5a76e4abf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f99bc3cce244267"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>